<commit_message>
MAIN 11 11 25
</commit_message>
<xml_diff>
--- a/Stat.xlsx
+++ b/Stat.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="105" windowWidth="27795" windowHeight="12345" activeTab="2"/>
+    <workbookView xWindow="360" yWindow="105" windowWidth="27795" windowHeight="12345" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -2114,6 +2114,13 @@
         <f t="shared" ref="B2:B34" si="0">IF(A2&lt;0, -1, IF(A2&gt;=3, 3, IF(A2&gt;=1, 0, "")))</f>
         <v>3</v>
       </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <f t="shared" ref="F2:F9" si="1">IF(E2&lt;0, -1, IF(E2&gt;=3, 3, IF(E2&gt;=1, 0, "")))</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3">
@@ -2123,6 +2130,13 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4">
@@ -2132,6 +2146,13 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
+      <c r="E4">
+        <v>-1</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="1"/>
+        <v>-1</v>
+      </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5">
@@ -2141,6 +2162,13 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="E5">
+        <v>-1</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="1"/>
+        <v>-1</v>
+      </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6">
@@ -2150,6 +2178,13 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="E6">
+        <v>-1</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="1"/>
+        <v>-1</v>
+      </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7">
@@ -2159,6 +2194,10 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
+      <c r="F7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8">
@@ -2168,6 +2207,10 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
+      <c r="F8" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9">
@@ -2177,6 +2220,10 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
+      <c r="F9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="10" spans="1:8">
       <c r="B10" t="str">
@@ -2201,14 +2248,14 @@
         <v>4</v>
       </c>
       <c r="E12" s="1">
-        <f t="shared" ref="E12:E32" si="1">IF(D12&lt;0, -1, IF(D12&gt;=3, 3, IF(D12&gt;=1, 0, "")))</f>
+        <f t="shared" ref="E12:E32" si="2">IF(D12&lt;0, -1, IF(D12&gt;=3, 3, IF(D12&gt;=1, 0, "")))</f>
         <v>3</v>
       </c>
       <c r="G12" s="1">
         <v>3</v>
       </c>
       <c r="H12" s="1">
-        <f t="shared" ref="H12:H32" si="2">IF(G12&lt;0, -1, IF(G12&gt;=3, 3, IF(G12&gt;=1, 0, "")))</f>
+        <f t="shared" ref="H12:H32" si="3">IF(G12&lt;0, -1, IF(G12&gt;=3, 3, IF(G12&gt;=1, 0, "")))</f>
         <v>3</v>
       </c>
     </row>
@@ -2224,14 +2271,14 @@
         <v>3</v>
       </c>
       <c r="E13" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="G13" s="1">
         <v>2</v>
       </c>
       <c r="H13" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2247,14 +2294,14 @@
         <v>8</v>
       </c>
       <c r="E14" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="G14" s="1">
         <v>1</v>
       </c>
       <c r="H14" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2270,14 +2317,14 @@
         <v>-1</v>
       </c>
       <c r="E15" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="G15" s="1">
         <v>-1</v>
       </c>
       <c r="H15" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-1</v>
       </c>
     </row>
@@ -2293,14 +2340,14 @@
         <v>-1</v>
       </c>
       <c r="E16" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="G16" s="1">
         <v>-1</v>
       </c>
       <c r="H16" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-1</v>
       </c>
     </row>
@@ -2316,14 +2363,14 @@
         <v>1</v>
       </c>
       <c r="E17" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G17" s="1">
         <v>2</v>
       </c>
       <c r="H17" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2339,14 +2386,14 @@
         <v>-1</v>
       </c>
       <c r="E18" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="G18" s="1">
         <v>-1</v>
       </c>
       <c r="H18" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-1</v>
       </c>
     </row>
@@ -2362,14 +2409,14 @@
         <v>-1</v>
       </c>
       <c r="E19" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="G19" s="1">
         <v>-1</v>
       </c>
       <c r="H19" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-1</v>
       </c>
     </row>
@@ -2385,14 +2432,14 @@
         <v>-1</v>
       </c>
       <c r="E20" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="G20" s="1">
         <v>4</v>
       </c>
       <c r="H20" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3</v>
       </c>
     </row>
@@ -2408,14 +2455,14 @@
         <v>4</v>
       </c>
       <c r="E21" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="G21" s="1">
         <v>3</v>
       </c>
       <c r="H21" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3</v>
       </c>
     </row>
@@ -2431,14 +2478,14 @@
         <v>3</v>
       </c>
       <c r="E22" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="G22" s="1">
         <v>3</v>
       </c>
       <c r="H22" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3</v>
       </c>
     </row>
@@ -2454,14 +2501,14 @@
         <v>4</v>
       </c>
       <c r="E23" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="G23" s="1">
         <v>3</v>
       </c>
       <c r="H23" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3</v>
       </c>
     </row>
@@ -2477,14 +2524,14 @@
         <v>-1</v>
       </c>
       <c r="E24" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="G24" s="1">
         <v>3</v>
       </c>
       <c r="H24" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3</v>
       </c>
     </row>
@@ -2500,14 +2547,14 @@
         <v>4</v>
       </c>
       <c r="E25" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="G25" s="1">
         <v>-1</v>
       </c>
       <c r="H25" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-1</v>
       </c>
     </row>
@@ -2523,12 +2570,12 @@
         <v>-1</v>
       </c>
       <c r="E26" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="G26" s="1"/>
       <c r="H26" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -2544,12 +2591,12 @@
         <v>4</v>
       </c>
       <c r="E27" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="G27" s="1"/>
       <c r="H27" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -2562,12 +2609,12 @@
         <v>1</v>
       </c>
       <c r="E28" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G28" s="1"/>
       <c r="H28" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -2579,12 +2626,12 @@
         <v>5</v>
       </c>
       <c r="E29" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="G29" s="1"/>
       <c r="H29" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -2600,12 +2647,12 @@
         <v>3</v>
       </c>
       <c r="E30" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="G30" s="1"/>
       <c r="H30" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -2621,12 +2668,12 @@
         <v>-1</v>
       </c>
       <c r="E31" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="G31" s="1"/>
       <c r="H31" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -2642,12 +2689,12 @@
         <v>3</v>
       </c>
       <c r="E32" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="G32" s="1"/>
       <c r="H32" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -2673,7 +2720,7 @@
     </row>
     <row r="36" spans="1:2">
       <c r="B36" t="str">
-        <f t="shared" ref="B36:B61" si="3">IF(A36&lt;0, -1, IF(A36&gt;=3, 3, IF(A36&gt;=1, 0, "")))</f>
+        <f t="shared" ref="B36:B61" si="4">IF(A36&lt;0, -1, IF(A36&gt;=3, 3, IF(A36&gt;=1, 0, "")))</f>
         <v/>
       </c>
     </row>
@@ -2682,7 +2729,7 @@
         <v>-1</v>
       </c>
       <c r="B37">
-        <f t="shared" ref="B37:B59" si="4">IF(A37&lt;0, -1, IF(A37&gt;=3, 3, IF(A37&gt;=1, 0, "")))</f>
+        <f t="shared" ref="B37:B59" si="5">IF(A37&lt;0, -1, IF(A37&gt;=3, 3, IF(A37&gt;=1, 0, "")))</f>
         <v>-1</v>
       </c>
     </row>
@@ -2691,7 +2738,7 @@
         <v>1</v>
       </c>
       <c r="B38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -2700,7 +2747,7 @@
         <v>5</v>
       </c>
       <c r="B39">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
     </row>
@@ -2709,7 +2756,7 @@
         <v>2.5</v>
       </c>
       <c r="B40">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -2718,7 +2765,7 @@
         <v>1</v>
       </c>
       <c r="B41">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -2727,7 +2774,7 @@
         <v>-1</v>
       </c>
       <c r="B42">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-1</v>
       </c>
     </row>
@@ -2736,7 +2783,7 @@
         <v>5</v>
       </c>
       <c r="B43">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
     </row>
@@ -2745,7 +2792,7 @@
         <v>5</v>
       </c>
       <c r="B44">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
     </row>
@@ -2754,7 +2801,7 @@
         <v>-1</v>
       </c>
       <c r="B45">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-1</v>
       </c>
     </row>
@@ -2763,7 +2810,7 @@
         <v>5</v>
       </c>
       <c r="B46">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
     </row>
@@ -2772,7 +2819,7 @@
         <v>4</v>
       </c>
       <c r="B47">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
     </row>
@@ -2781,7 +2828,7 @@
         <v>3</v>
       </c>
       <c r="B48">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
     </row>
@@ -2790,7 +2837,7 @@
         <v>3</v>
       </c>
       <c r="B49">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
     </row>
@@ -2799,7 +2846,7 @@
         <v>-1</v>
       </c>
       <c r="B50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-1</v>
       </c>
     </row>
@@ -2808,7 +2855,7 @@
         <v>-1</v>
       </c>
       <c r="B51">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-1</v>
       </c>
     </row>
@@ -2817,7 +2864,7 @@
         <v>4</v>
       </c>
       <c r="B52">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
     </row>
@@ -2826,7 +2873,7 @@
         <v>-1</v>
       </c>
       <c r="B53">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-1</v>
       </c>
     </row>
@@ -2835,37 +2882,37 @@
         <v>-1</v>
       </c>
       <c r="B54">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>-1</v>
       </c>
     </row>
     <row r="55" spans="1:9">
       <c r="B55" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="56" spans="1:9">
       <c r="B56" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="57" spans="1:9">
       <c r="B57" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="58" spans="1:9">
       <c r="B58" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="59" spans="1:9">
       <c r="B59" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2874,25 +2921,25 @@
         <v>7</v>
       </c>
       <c r="I60" t="str">
-        <f t="shared" ref="I60" si="5">IF(H60&lt;0, -1, IF(H60&gt;=3, 3, IF(H60&gt;=1, 0, "")))</f>
+        <f t="shared" ref="I60" si="6">IF(H60&lt;0, -1, IF(H60&gt;=3, 3, IF(H60&gt;=1, 0, "")))</f>
         <v/>
       </c>
     </row>
     <row r="61" spans="1:9">
       <c r="B61" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
     <row r="62" spans="1:9">
       <c r="B62" t="str">
-        <f t="shared" ref="B62:B125" si="6">IF(A62&lt;0, -1, IF(A62&gt;=3, 3, IF(A62&gt;=1, 0, "")))</f>
+        <f t="shared" ref="B62:B125" si="7">IF(A62&lt;0, -1, IF(A62&gt;=3, 3, IF(A62&gt;=1, 0, "")))</f>
         <v/>
       </c>
     </row>
     <row r="63" spans="1:9">
       <c r="B63" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -2901,7 +2948,7 @@
         <v>-1</v>
       </c>
       <c r="B64">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-1</v>
       </c>
     </row>
@@ -2910,7 +2957,7 @@
         <v>-1</v>
       </c>
       <c r="B65">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-1</v>
       </c>
     </row>
@@ -2919,7 +2966,7 @@
         <v>4</v>
       </c>
       <c r="B66">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
     </row>
@@ -2928,7 +2975,7 @@
         <v>2</v>
       </c>
       <c r="B67">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -2937,7 +2984,7 @@
         <v>-1</v>
       </c>
       <c r="B68">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-1</v>
       </c>
     </row>
@@ -2946,7 +2993,7 @@
         <v>5</v>
       </c>
       <c r="B69">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
     </row>
@@ -2955,7 +3002,7 @@
         <v>5</v>
       </c>
       <c r="B70">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
     </row>
@@ -2964,7 +3011,7 @@
         <v>-1</v>
       </c>
       <c r="B71">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-1</v>
       </c>
     </row>
@@ -2973,7 +3020,7 @@
         <v>5</v>
       </c>
       <c r="B72">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
     </row>
@@ -2982,7 +3029,7 @@
         <v>-1</v>
       </c>
       <c r="B73">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-1</v>
       </c>
     </row>
@@ -2991,7 +3038,7 @@
         <v>3</v>
       </c>
       <c r="B74">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
     </row>
@@ -3000,7 +3047,7 @@
         <v>-1</v>
       </c>
       <c r="B75">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-1</v>
       </c>
     </row>
@@ -3009,7 +3056,7 @@
         <v>3</v>
       </c>
       <c r="B76">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
     </row>
@@ -3018,7 +3065,7 @@
         <v>1</v>
       </c>
       <c r="B77">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -3027,7 +3074,7 @@
         <v>4</v>
       </c>
       <c r="B78">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
     </row>
@@ -3036,7 +3083,7 @@
         <v>1</v>
       </c>
       <c r="B79">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -3045,7 +3092,7 @@
         <v>-1</v>
       </c>
       <c r="B80">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-1</v>
       </c>
     </row>
@@ -3054,7 +3101,7 @@
         <v>-1</v>
       </c>
       <c r="B81">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-1</v>
       </c>
     </row>
@@ -3063,7 +3110,7 @@
         <v>5</v>
       </c>
       <c r="B82">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
     </row>
@@ -3072,7 +3119,7 @@
         <v>-1</v>
       </c>
       <c r="B83">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-1</v>
       </c>
     </row>
@@ -3081,25 +3128,25 @@
         <v>3</v>
       </c>
       <c r="B84">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="B85" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="B86" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="B87" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -3113,7 +3160,7 @@
         <v>4</v>
       </c>
       <c r="B89">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
     </row>
@@ -3122,7 +3169,7 @@
         <v>5</v>
       </c>
       <c r="B90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
     </row>
@@ -3131,7 +3178,7 @@
         <v>5</v>
       </c>
       <c r="B91">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
     </row>
@@ -3140,7 +3187,7 @@
         <v>-1</v>
       </c>
       <c r="B92">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-1</v>
       </c>
     </row>
@@ -3149,7 +3196,7 @@
         <v>4</v>
       </c>
       <c r="B93">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
     </row>
@@ -3158,7 +3205,7 @@
         <v>-1</v>
       </c>
       <c r="B94">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-1</v>
       </c>
     </row>
@@ -3167,7 +3214,7 @@
         <v>-1</v>
       </c>
       <c r="B95">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-1</v>
       </c>
     </row>
@@ -3176,7 +3223,7 @@
         <v>4</v>
       </c>
       <c r="B96">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
     </row>
@@ -3185,985 +3232,985 @@
         <v>4</v>
       </c>
       <c r="B97">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="B98" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="B99" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="B100" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="B101" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="B102" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="B103" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="B104" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="B105" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="B106" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="B107" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="B108" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="B109" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="B110" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="B111" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="B112" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="113" spans="2:2">
       <c r="B113" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="114" spans="2:2">
       <c r="B114" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="115" spans="2:2">
       <c r="B115" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="116" spans="2:2">
       <c r="B116" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="117" spans="2:2">
       <c r="B117" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="118" spans="2:2">
       <c r="B118" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="119" spans="2:2">
       <c r="B119" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="120" spans="2:2">
       <c r="B120" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="121" spans="2:2">
       <c r="B121" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="122" spans="2:2">
       <c r="B122" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="123" spans="2:2">
       <c r="B123" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="124" spans="2:2">
       <c r="B124" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="125" spans="2:2">
       <c r="B125" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="126" spans="2:2">
       <c r="B126" t="str">
-        <f t="shared" ref="B126:B189" si="7">IF(A126&lt;0, -1, IF(A126&gt;=3, 3, IF(A126&gt;=1, 0, "")))</f>
+        <f t="shared" ref="B126:B189" si="8">IF(A126&lt;0, -1, IF(A126&gt;=3, 3, IF(A126&gt;=1, 0, "")))</f>
         <v/>
       </c>
     </row>
     <row r="127" spans="2:2">
       <c r="B127" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="128" spans="2:2">
       <c r="B128" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="129" spans="2:2">
       <c r="B129" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="130" spans="2:2">
       <c r="B130" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="131" spans="2:2">
       <c r="B131" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="132" spans="2:2">
       <c r="B132" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="133" spans="2:2">
       <c r="B133" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="134" spans="2:2">
       <c r="B134" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="135" spans="2:2">
       <c r="B135" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="136" spans="2:2">
       <c r="B136" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="137" spans="2:2">
       <c r="B137" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="138" spans="2:2">
       <c r="B138" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="139" spans="2:2">
       <c r="B139" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="140" spans="2:2">
       <c r="B140" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="141" spans="2:2">
       <c r="B141" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="142" spans="2:2">
       <c r="B142" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="143" spans="2:2">
       <c r="B143" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="144" spans="2:2">
       <c r="B144" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="145" spans="2:2">
       <c r="B145" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="146" spans="2:2">
       <c r="B146" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="147" spans="2:2">
       <c r="B147" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="148" spans="2:2">
       <c r="B148" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="149" spans="2:2">
       <c r="B149" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="150" spans="2:2">
       <c r="B150" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="151" spans="2:2">
       <c r="B151" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="152" spans="2:2">
       <c r="B152" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="153" spans="2:2">
       <c r="B153" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="154" spans="2:2">
       <c r="B154" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="155" spans="2:2">
       <c r="B155" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="156" spans="2:2">
       <c r="B156" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="157" spans="2:2">
       <c r="B157" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="158" spans="2:2">
       <c r="B158" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="159" spans="2:2">
       <c r="B159" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="160" spans="2:2">
       <c r="B160" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="161" spans="2:2">
       <c r="B161" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="162" spans="2:2">
       <c r="B162" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="163" spans="2:2">
       <c r="B163" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="164" spans="2:2">
       <c r="B164" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="165" spans="2:2">
       <c r="B165" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="166" spans="2:2">
       <c r="B166" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="167" spans="2:2">
       <c r="B167" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="168" spans="2:2">
       <c r="B168" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="169" spans="2:2">
       <c r="B169" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="170" spans="2:2">
       <c r="B170" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="171" spans="2:2">
       <c r="B171" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="172" spans="2:2">
       <c r="B172" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="173" spans="2:2">
       <c r="B173" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="174" spans="2:2">
       <c r="B174" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="175" spans="2:2">
       <c r="B175" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="176" spans="2:2">
       <c r="B176" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="177" spans="2:2">
       <c r="B177" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="178" spans="2:2">
       <c r="B178" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="179" spans="2:2">
       <c r="B179" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="180" spans="2:2">
       <c r="B180" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="181" spans="2:2">
       <c r="B181" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="182" spans="2:2">
       <c r="B182" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="183" spans="2:2">
       <c r="B183" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="184" spans="2:2">
       <c r="B184" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="185" spans="2:2">
       <c r="B185" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="186" spans="2:2">
       <c r="B186" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="187" spans="2:2">
       <c r="B187" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="188" spans="2:2">
       <c r="B188" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="189" spans="2:2">
       <c r="B189" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="190" spans="2:2">
       <c r="B190" t="str">
-        <f t="shared" ref="B190:B200" si="8">IF(A190&lt;0, -1, IF(A190&gt;=3, 3, IF(A190&gt;=1, 0, "")))</f>
+        <f t="shared" ref="B190:B200" si="9">IF(A190&lt;0, -1, IF(A190&gt;=3, 3, IF(A190&gt;=1, 0, "")))</f>
         <v/>
       </c>
     </row>
     <row r="191" spans="2:2">
       <c r="B191" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
     </row>
     <row r="192" spans="2:2">
       <c r="B192" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
     </row>
     <row r="193" spans="2:2">
       <c r="B193" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
     </row>
     <row r="194" spans="2:2">
       <c r="B194" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
     </row>
     <row r="195" spans="2:2">
       <c r="B195" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
     </row>
     <row r="196" spans="2:2">
       <c r="B196" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
     </row>
     <row r="197" spans="2:2">
       <c r="B197" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
     </row>
     <row r="198" spans="2:2">
       <c r="B198" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
     </row>
     <row r="199" spans="2:2">
       <c r="B199" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
     </row>
     <row r="200" spans="2:2">
       <c r="B200" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
     </row>
     <row r="201" spans="2:2">
       <c r="B201" t="str">
-        <f t="shared" ref="B201:B223" si="9">IF(A201&lt;0, -1, IF(A201&gt;=3, 3, IF(A201&gt;=1, 0, "")))</f>
+        <f t="shared" ref="B201:B223" si="10">IF(A201&lt;0, -1, IF(A201&gt;=3, 3, IF(A201&gt;=1, 0, "")))</f>
         <v/>
       </c>
     </row>
     <row r="202" spans="2:2">
       <c r="B202" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="203" spans="2:2">
       <c r="B203" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="204" spans="2:2">
       <c r="B204" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="205" spans="2:2">
       <c r="B205" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="206" spans="2:2">
       <c r="B206" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="207" spans="2:2">
       <c r="B207" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="208" spans="2:2">
       <c r="B208" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="209" spans="2:2">
       <c r="B209" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="210" spans="2:2">
       <c r="B210" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="211" spans="2:2">
       <c r="B211" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="212" spans="2:2">
       <c r="B212" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="213" spans="2:2">
       <c r="B213" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="214" spans="2:2">
       <c r="B214" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="215" spans="2:2">
       <c r="B215" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="216" spans="2:2">
       <c r="B216" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="217" spans="2:2">
       <c r="B217" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="218" spans="2:2">
       <c r="B218" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="219" spans="2:2">
       <c r="B219" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="220" spans="2:2">
       <c r="B220" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="221" spans="2:2">
       <c r="B221" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="222" spans="2:2">
       <c r="B222" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="223" spans="2:2">
       <c r="B223" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="224" spans="2:2">
       <c r="B224" t="str">
-        <f t="shared" ref="B224:B260" si="10">IF(A224&lt;0, -1, IF(A224&gt;=3, 3, IF(A224&gt;=1, 0, "")))</f>
+        <f t="shared" ref="B224:B260" si="11">IF(A224&lt;0, -1, IF(A224&gt;=3, 3, IF(A224&gt;=1, 0, "")))</f>
         <v/>
       </c>
     </row>
     <row r="225" spans="2:2">
       <c r="B225" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="226" spans="2:2">
       <c r="B226" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="227" spans="2:2">
       <c r="B227" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="228" spans="2:2">
       <c r="B228" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="229" spans="2:2">
       <c r="B229" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="230" spans="2:2">
       <c r="B230" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="231" spans="2:2">
       <c r="B231" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="232" spans="2:2">
       <c r="B232" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="233" spans="2:2">
       <c r="B233" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="234" spans="2:2">
       <c r="B234" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="235" spans="2:2">
       <c r="B235" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="236" spans="2:2">
       <c r="B236" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="237" spans="2:2">
       <c r="B237" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="238" spans="2:2">
       <c r="B238" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="239" spans="2:2">
       <c r="B239" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="240" spans="2:2">
       <c r="B240" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="241" spans="2:2">
       <c r="B241" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="242" spans="2:2">
       <c r="B242" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="243" spans="2:2">
       <c r="B243" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="244" spans="2:2">
       <c r="B244" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="245" spans="2:2">
       <c r="B245" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="246" spans="2:2">
       <c r="B246" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="247" spans="2:2">
       <c r="B247" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="248" spans="2:2">
       <c r="B248" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="249" spans="2:2">
       <c r="B249" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="250" spans="2:2">
       <c r="B250" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="251" spans="2:2">
       <c r="B251" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="252" spans="2:2">
       <c r="B252" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="253" spans="2:2">
       <c r="B253" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="254" spans="2:2">
       <c r="B254" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="255" spans="2:2">
       <c r="B255" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="256" spans="2:2">
       <c r="B256" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="257" spans="2:2">
       <c r="B257" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="258" spans="2:2">
       <c r="B258" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="259" spans="2:2">
       <c r="B259" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="260" spans="2:2">
       <c r="B260" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
@@ -4288,7 +4335,7 @@
         <v>3</v>
       </c>
       <c r="B21" s="1">
-        <f t="shared" ref="B21:B40" si="1">IF(A21&lt;0, -1, IF(A21&gt;=3, 3, IF(A21&gt;=1, 0, "")))</f>
+        <f t="shared" ref="B21:B39" si="1">IF(A21&lt;0, -1, IF(A21&gt;=3, 3, IF(A21&gt;=1, 0, "")))</f>
         <v>3</v>
       </c>
     </row>
@@ -4879,7 +4926,7 @@
         <v>2</v>
       </c>
       <c r="E110">
-        <f t="shared" ref="E110:E144" si="4">IF(D110&lt;0, -1, IF(D110&gt;=3, 3, IF(D110&gt;=1, 0, "")))</f>
+        <f t="shared" ref="E110:E119" si="4">IF(D110&lt;0, -1, IF(D110&gt;=3, 3, IF(D110&gt;=1, 0, "")))</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>